<commit_message>
fast model analysis skim
</commit_message>
<xml_diff>
--- a/artifacts/analysis/model-analysis.xlsx
+++ b/artifacts/analysis/model-analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jn\dev\llm-ensemble\artifacts\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{264E60F2-587C-4EC3-8CDA-A0DCB68656EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B90D2B1-D362-4C83-9342-50BEE56CAF6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{D1A87F95-65CE-44FE-B65A-B20AE0988E6A}"/>
   </bookViews>
@@ -566,18 +566,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -637,12 +631,6 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="27" formatCode="m/d/yyyy\ h:mm"/>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -711,6 +699,12 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
@@ -756,53 +750,53 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E74BC6F4-E459-4841-A57F-F7392AD4352B}" name="models_202601091237" displayName="models_202601091237" ref="A1:T16" tableType="queryTable" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E74BC6F4-E459-4841-A57F-F7392AD4352B}" name="models_202601091237" displayName="models_202601091237" ref="A1:T16" tableType="queryTable" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <autoFilter ref="A1:T16" xr:uid="{E74BC6F4-E459-4841-A57F-F7392AD4352B}"/>
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{78D3B969-8519-472B-B7DC-40B2AB389EDF}" uniqueName="1" name="model_id" queryTableFieldId="1" dataDxfId="38"/>
-    <tableColumn id="2" xr3:uid="{2775870E-97E4-4A13-8631-08858414ABE9}" uniqueName="2" name="canonical_slug" queryTableFieldId="2" dataDxfId="37"/>
-    <tableColumn id="3" xr3:uid="{9123C448-65CD-42A3-A8DF-FA33362CF2EB}" uniqueName="3" name="model_name" queryTableFieldId="3" dataDxfId="36"/>
-    <tableColumn id="4" xr3:uid="{23ACEE67-B62B-4941-8C62-48ACD4FFD384}" uniqueName="4" name="description" queryTableFieldId="4" dataDxfId="35"/>
-    <tableColumn id="5" xr3:uid="{EBBFCEC0-7D31-4CAD-A2DD-E444E8C840AD}" uniqueName="5" name="created" queryTableFieldId="5" dataDxfId="34"/>
-    <tableColumn id="6" xr3:uid="{235BBD11-52A4-432B-B259-1FEF7849A476}" uniqueName="6" name="prompt_cost_per_1m" queryTableFieldId="6" dataDxfId="33"/>
-    <tableColumn id="7" xr3:uid="{C125A326-71DC-498F-9CF6-9D4261986ABF}" uniqueName="7" name="completion_cost_per_1m" queryTableFieldId="7" dataDxfId="32"/>
-    <tableColumn id="8" xr3:uid="{C48D515D-EA76-4B8D-9D9B-3F86005C986D}" uniqueName="8" name="avg_cost_per_1m" queryTableFieldId="8" dataDxfId="31"/>
-    <tableColumn id="9" xr3:uid="{0C9AC00E-B68D-4AF7-9758-7543FA934B04}" uniqueName="9" name="request_cost" queryTableFieldId="9" dataDxfId="30"/>
-    <tableColumn id="10" xr3:uid="{CED2343B-816C-4F54-B994-E7FC118F7157}" uniqueName="10" name="image_cost" queryTableFieldId="10" dataDxfId="29"/>
-    <tableColumn id="11" xr3:uid="{6D67746F-12ED-4C55-AF34-2427D5CEA21F}" uniqueName="11" name="is_free" queryTableFieldId="11" dataDxfId="28"/>
-    <tableColumn id="12" xr3:uid="{D41C5152-EBB5-4D0D-A3D0-E2AF2584030A}" uniqueName="12" name="param_size" queryTableFieldId="12" dataDxfId="27"/>
-    <tableColumn id="13" xr3:uid="{3F7A75A1-5B17-4021-B0DF-2D6D58413453}" uniqueName="13" name="context_length" queryTableFieldId="13" dataDxfId="26"/>
-    <tableColumn id="14" xr3:uid="{77302B12-EFD5-4388-8BAA-BE5B0C3E0D4D}" uniqueName="14" name="architecture" queryTableFieldId="14" dataDxfId="25"/>
-    <tableColumn id="15" xr3:uid="{A4F53FD9-655C-485A-AF2A-687B004D91BB}" uniqueName="15" name="top_provider" queryTableFieldId="15" dataDxfId="24"/>
-    <tableColumn id="16" xr3:uid="{8DC3E8E9-B9CD-4A00-ABDC-CAEB3EF2F82E}" uniqueName="16" name="per_request_limits" queryTableFieldId="16" dataDxfId="23"/>
-    <tableColumn id="17" xr3:uid="{89C9A0EC-EEDE-4BF2-9AD6-BFB8C497DC96}" uniqueName="17" name="supported_parameters" queryTableFieldId="17" dataDxfId="22"/>
-    <tableColumn id="18" xr3:uid="{782F3ED8-5B9C-4F0A-9BF7-C9083C418B46}" uniqueName="18" name="default_parameters" queryTableFieldId="18" dataDxfId="21"/>
-    <tableColumn id="19" xr3:uid="{B52B03E2-D483-4B78-B500-90C21984E5CF}" uniqueName="19" name="last_updated" queryTableFieldId="19" dataDxfId="20"/>
-    <tableColumn id="20" xr3:uid="{A9E6322E-6414-4705-8C48-2E513F4761A1}" uniqueName="20" name="created_at" queryTableFieldId="20" dataDxfId="19"/>
+    <tableColumn id="1" xr3:uid="{78D3B969-8519-472B-B7DC-40B2AB389EDF}" uniqueName="1" name="model_id" queryTableFieldId="1" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{2775870E-97E4-4A13-8631-08858414ABE9}" uniqueName="2" name="canonical_slug" queryTableFieldId="2" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{9123C448-65CD-42A3-A8DF-FA33362CF2EB}" uniqueName="3" name="model_name" queryTableFieldId="3" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{23ACEE67-B62B-4941-8C62-48ACD4FFD384}" uniqueName="4" name="description" queryTableFieldId="4" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{EBBFCEC0-7D31-4CAD-A2DD-E444E8C840AD}" uniqueName="5" name="created" queryTableFieldId="5" dataDxfId="32"/>
+    <tableColumn id="6" xr3:uid="{235BBD11-52A4-432B-B259-1FEF7849A476}" uniqueName="6" name="prompt_cost_per_1m" queryTableFieldId="6" dataDxfId="31"/>
+    <tableColumn id="7" xr3:uid="{C125A326-71DC-498F-9CF6-9D4261986ABF}" uniqueName="7" name="completion_cost_per_1m" queryTableFieldId="7" dataDxfId="30"/>
+    <tableColumn id="8" xr3:uid="{C48D515D-EA76-4B8D-9D9B-3F86005C986D}" uniqueName="8" name="avg_cost_per_1m" queryTableFieldId="8" dataDxfId="29"/>
+    <tableColumn id="9" xr3:uid="{0C9AC00E-B68D-4AF7-9758-7543FA934B04}" uniqueName="9" name="request_cost" queryTableFieldId="9" dataDxfId="28"/>
+    <tableColumn id="10" xr3:uid="{CED2343B-816C-4F54-B994-E7FC118F7157}" uniqueName="10" name="image_cost" queryTableFieldId="10" dataDxfId="27"/>
+    <tableColumn id="11" xr3:uid="{6D67746F-12ED-4C55-AF34-2427D5CEA21F}" uniqueName="11" name="is_free" queryTableFieldId="11" dataDxfId="26"/>
+    <tableColumn id="12" xr3:uid="{D41C5152-EBB5-4D0D-A3D0-E2AF2584030A}" uniqueName="12" name="param_size" queryTableFieldId="12" dataDxfId="25"/>
+    <tableColumn id="13" xr3:uid="{3F7A75A1-5B17-4021-B0DF-2D6D58413453}" uniqueName="13" name="context_length" queryTableFieldId="13" dataDxfId="24"/>
+    <tableColumn id="14" xr3:uid="{77302B12-EFD5-4388-8BAA-BE5B0C3E0D4D}" uniqueName="14" name="architecture" queryTableFieldId="14" dataDxfId="23"/>
+    <tableColumn id="15" xr3:uid="{A4F53FD9-655C-485A-AF2A-687B004D91BB}" uniqueName="15" name="top_provider" queryTableFieldId="15" dataDxfId="22"/>
+    <tableColumn id="16" xr3:uid="{8DC3E8E9-B9CD-4A00-ABDC-CAEB3EF2F82E}" uniqueName="16" name="per_request_limits" queryTableFieldId="16" dataDxfId="21"/>
+    <tableColumn id="17" xr3:uid="{89C9A0EC-EEDE-4BF2-9AD6-BFB8C497DC96}" uniqueName="17" name="supported_parameters" queryTableFieldId="17" dataDxfId="20"/>
+    <tableColumn id="18" xr3:uid="{782F3ED8-5B9C-4F0A-9BF7-C9083C418B46}" uniqueName="18" name="default_parameters" queryTableFieldId="18" dataDxfId="19"/>
+    <tableColumn id="19" xr3:uid="{B52B03E2-D483-4B78-B500-90C21984E5CF}" uniqueName="19" name="last_updated" queryTableFieldId="19" dataDxfId="18"/>
+    <tableColumn id="20" xr3:uid="{A9E6322E-6414-4705-8C48-2E513F4761A1}" uniqueName="20" name="created_at" queryTableFieldId="20" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2515506D-7B69-4B06-9BF5-773B122E6626}" name="Table6" displayName="Table6" ref="A1:O16" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2515506D-7B69-4B06-9BF5-773B122E6626}" name="Table6" displayName="Table6" ref="A1:O16" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A1:O16" xr:uid="{2515506D-7B69-4B06-9BF5-773B122E6626}"/>
   <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{D58B9424-3D3A-43E3-A095-F707C822ADC7}" name="model_id" dataDxfId="16" dataCellStyle="Normal"/>
-    <tableColumn id="2" xr3:uid="{00B31618-54C8-49F9-A9FF-AA301F6B83EE}" name="provider" dataDxfId="15" dataCellStyle="Normal"/>
-    <tableColumn id="15" xr3:uid="{B2A402DF-F928-46BF-A6E6-444AE9EAEC05}" name="Location" dataDxfId="14"/>
-    <tableColumn id="3" xr3:uid="{FB0B91F9-CC4A-4F2F-B7FA-8F4849679D55}" name="training data" dataDxfId="13" dataCellStyle="Normal"/>
-    <tableColumn id="4" xr3:uid="{710908A7-2136-47EA-9EA4-61FB50EB1236}" name="Input modalities" dataDxfId="12" dataCellStyle="Normal"/>
-    <tableColumn id="5" xr3:uid="{E231CFF8-225F-4DDB-B084-555A9DCA2D9B}" name="Output modalities" dataDxfId="11" dataCellStyle="Normal"/>
-    <tableColumn id="6" xr3:uid="{97A650FA-812C-420D-8844-FAB2DDACEEE8}" name="Architecture" dataDxfId="10" dataCellStyle="Normal"/>
-    <tableColumn id="7" xr3:uid="{ACE0B5AB-F0DE-44AF-BDA1-3D7933AA8AF9}" name="Reasoning" dataDxfId="9" dataCellStyle="Normal"/>
-    <tableColumn id="8" xr3:uid="{81A13497-D9E5-4952-BA69-5ECB2716882B}" name="Optimized For" dataDxfId="8" dataCellStyle="Normal"/>
-    <tableColumn id="9" xr3:uid="{2050FC21-8B57-4EC1-AF1A-DAECC9F9B2CB}" name="Alignment" dataDxfId="7" dataCellStyle="Normal"/>
-    <tableColumn id="10" xr3:uid="{CB6C60B6-16A5-463B-99B4-39EA4C602AD1}" name="average cost per million token" dataDxfId="6" dataCellStyle="Normal"/>
-    <tableColumn id="11" xr3:uid="{EFDCD220-B721-413F-9910-7C191803D101}" name="cost tier" dataDxfId="5" dataCellStyle="Normal"/>
-    <tableColumn id="12" xr3:uid="{2143AF97-E365-40D2-8B0E-2F9755C0F893}" name="openrouter link" dataDxfId="4" dataCellStyle="Normal"/>
-    <tableColumn id="13" xr3:uid="{0516A28C-43F7-4683-AB8C-D7BCE4C57A35}" name="other links" dataDxfId="3" dataCellStyle="Normal"/>
-    <tableColumn id="14" xr3:uid="{84069568-AA3D-4C3F-98FC-E07C771A4615}" name="Column1" dataDxfId="2" dataCellStyle="Normal"/>
+    <tableColumn id="1" xr3:uid="{D58B9424-3D3A-43E3-A095-F707C822ADC7}" name="model_id" dataDxfId="14" dataCellStyle="Normal"/>
+    <tableColumn id="2" xr3:uid="{00B31618-54C8-49F9-A9FF-AA301F6B83EE}" name="provider" dataDxfId="13" dataCellStyle="Normal"/>
+    <tableColumn id="15" xr3:uid="{B2A402DF-F928-46BF-A6E6-444AE9EAEC05}" name="Location" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{FB0B91F9-CC4A-4F2F-B7FA-8F4849679D55}" name="training data" dataDxfId="11" dataCellStyle="Normal"/>
+    <tableColumn id="4" xr3:uid="{710908A7-2136-47EA-9EA4-61FB50EB1236}" name="Input modalities" dataDxfId="10" dataCellStyle="Normal"/>
+    <tableColumn id="5" xr3:uid="{E231CFF8-225F-4DDB-B084-555A9DCA2D9B}" name="Output modalities" dataDxfId="9" dataCellStyle="Normal"/>
+    <tableColumn id="6" xr3:uid="{97A650FA-812C-420D-8844-FAB2DDACEEE8}" name="Architecture" dataDxfId="8" dataCellStyle="Normal"/>
+    <tableColumn id="7" xr3:uid="{ACE0B5AB-F0DE-44AF-BDA1-3D7933AA8AF9}" name="Reasoning" dataDxfId="7" dataCellStyle="Normal"/>
+    <tableColumn id="8" xr3:uid="{81A13497-D9E5-4952-BA69-5ECB2716882B}" name="Optimized For" dataDxfId="6" dataCellStyle="Normal"/>
+    <tableColumn id="9" xr3:uid="{2050FC21-8B57-4EC1-AF1A-DAECC9F9B2CB}" name="Alignment" dataDxfId="5" dataCellStyle="Normal"/>
+    <tableColumn id="10" xr3:uid="{CB6C60B6-16A5-463B-99B4-39EA4C602AD1}" name="average cost per million token" dataDxfId="4" dataCellStyle="Normal"/>
+    <tableColumn id="11" xr3:uid="{EFDCD220-B721-413F-9910-7C191803D101}" name="cost tier" dataDxfId="3" dataCellStyle="Normal"/>
+    <tableColumn id="12" xr3:uid="{2143AF97-E365-40D2-8B0E-2F9755C0F893}" name="openrouter link" dataDxfId="2" dataCellStyle="Normal"/>
+    <tableColumn id="13" xr3:uid="{0516A28C-43F7-4683-AB8C-D7BCE4C57A35}" name="other links" dataDxfId="1" dataCellStyle="Normal"/>
+    <tableColumn id="14" xr3:uid="{84069568-AA3D-4C3F-98FC-E07C771A4615}" name="Column1" dataDxfId="0" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1213,16 +1207,16 @@
       </c>
     </row>
     <row r="2" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="1" t="s">
         <v>70</v>
       </c>
       <c r="E2" s="1">
@@ -1252,39 +1246,39 @@
       <c r="M2" s="1">
         <v>128000</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="O2" s="2" t="s">
+      <c r="O2" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="P2" s="2" t="s">
+      <c r="P2" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q2" s="2" t="s">
+      <c r="Q2" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="R2" s="2" t="s">
+      <c r="R2" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="S2" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T2" s="3">
+      <c r="S2" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T2" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="3" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="1" t="s">
         <v>75</v>
       </c>
       <c r="E3" s="1">
@@ -1314,39 +1308,39 @@
       <c r="M3" s="1">
         <v>128000</v>
       </c>
-      <c r="N3" s="2" t="s">
+      <c r="N3" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="O3" s="2" t="s">
+      <c r="O3" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="P3" s="2" t="s">
+      <c r="P3" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q3" s="2" t="s">
+      <c r="Q3" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="R3" s="2" t="s">
+      <c r="R3" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="S3" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T3" s="3">
+      <c r="S3" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T3" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="4" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="1" t="s">
         <v>79</v>
       </c>
       <c r="E4" s="1">
@@ -1376,39 +1370,39 @@
       <c r="M4" s="1">
         <v>128000</v>
       </c>
-      <c r="N4" s="2" t="s">
+      <c r="N4" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="O4" s="2" t="s">
+      <c r="O4" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="P4" s="2" t="s">
+      <c r="P4" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q4" s="2" t="s">
+      <c r="Q4" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="R4" s="2" t="s">
+      <c r="R4" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="S4" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T4" s="3">
+      <c r="S4" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T4" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="5" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="1" t="s">
         <v>84</v>
       </c>
       <c r="E5" s="1">
@@ -1438,39 +1432,39 @@
       <c r="M5" s="1">
         <v>96000</v>
       </c>
-      <c r="N5" s="2" t="s">
+      <c r="N5" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="O5" s="2" t="s">
+      <c r="O5" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="P5" s="2" t="s">
+      <c r="P5" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q5" s="2" t="s">
+      <c r="Q5" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="R5" s="2" t="s">
+      <c r="R5" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="S5" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T5" s="3">
+      <c r="S5" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T5" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="6" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="1" t="s">
         <v>88</v>
       </c>
       <c r="E6" s="1">
@@ -1500,39 +1494,39 @@
       <c r="M6" s="1">
         <v>131000</v>
       </c>
-      <c r="N6" s="2" t="s">
+      <c r="N6" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="O6" s="2" t="s">
+      <c r="O6" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="P6" s="2" t="s">
+      <c r="P6" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q6" s="2" t="s">
+      <c r="Q6" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="R6" s="2" t="s">
+      <c r="R6" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="S6" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T6" s="3">
+      <c r="S6" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T6" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="7" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="2" t="s">
+      <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="2" t="s">
+      <c r="D7" s="1" t="s">
         <v>92</v>
       </c>
       <c r="E7" s="1">
@@ -1562,39 +1556,39 @@
       <c r="M7" s="1">
         <v>131072</v>
       </c>
-      <c r="N7" s="2" t="s">
+      <c r="N7" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="O7" s="2" t="s">
+      <c r="O7" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="P7" s="2" t="s">
+      <c r="P7" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q7" s="2" t="s">
+      <c r="Q7" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="R7" s="2" t="s">
+      <c r="R7" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="S7" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T7" s="3">
+      <c r="S7" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T7" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="8" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="2" t="s">
+      <c r="A8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="1" t="s">
         <v>95</v>
       </c>
       <c r="E8" s="1">
@@ -1624,39 +1618,39 @@
       <c r="M8" s="1">
         <v>131072</v>
       </c>
-      <c r="N8" s="2" t="s">
+      <c r="N8" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="O8" s="2" t="s">
+      <c r="O8" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="P8" s="2" t="s">
+      <c r="P8" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q8" s="2" t="s">
+      <c r="Q8" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="R8" s="2" t="s">
+      <c r="R8" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="S8" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T8" s="3">
+      <c r="S8" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T8" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="9" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="1" t="s">
         <v>99</v>
       </c>
       <c r="E9" s="1">
@@ -1686,39 +1680,39 @@
       <c r="M9" s="1">
         <v>131072</v>
       </c>
-      <c r="N9" s="2" t="s">
+      <c r="N9" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="O9" s="2" t="s">
+      <c r="O9" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="P9" s="2" t="s">
+      <c r="P9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q9" s="2" t="s">
+      <c r="Q9" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="R9" s="2" t="s">
+      <c r="R9" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="S9" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T9" s="3">
+      <c r="S9" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T9" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="10" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="1" t="s">
         <v>101</v>
       </c>
       <c r="E10" s="1">
@@ -1748,39 +1742,39 @@
       <c r="M10" s="1">
         <v>131072</v>
       </c>
-      <c r="N10" s="2" t="s">
+      <c r="N10" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="O10" s="2" t="s">
+      <c r="O10" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="P10" s="2" t="s">
+      <c r="P10" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q10" s="2" t="s">
+      <c r="Q10" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="R10" s="2" t="s">
+      <c r="R10" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="S10" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T10" s="3">
+      <c r="S10" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T10" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="11" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="2" t="s">
+      <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="2" t="s">
+      <c r="D11" s="1" t="s">
         <v>105</v>
       </c>
       <c r="E11" s="1">
@@ -1810,39 +1804,39 @@
       <c r="M11" s="1">
         <v>262144</v>
       </c>
-      <c r="N11" s="2" t="s">
+      <c r="N11" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="O11" s="2" t="s">
+      <c r="O11" s="1" t="s">
         <v>106</v>
       </c>
-      <c r="P11" s="2" t="s">
+      <c r="P11" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q11" s="2" t="s">
+      <c r="Q11" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="R11" s="2" t="s">
+      <c r="R11" s="1" t="s">
         <v>104</v>
       </c>
-      <c r="S11" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T11" s="3">
+      <c r="S11" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T11" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="12" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="2" t="s">
+      <c r="D12" s="1" t="s">
         <v>107</v>
       </c>
       <c r="E12" s="1">
@@ -1872,39 +1866,39 @@
       <c r="M12" s="1">
         <v>131072</v>
       </c>
-      <c r="N12" s="2" t="s">
+      <c r="N12" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="O12" s="2" t="s">
+      <c r="O12" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="P12" s="2" t="s">
+      <c r="P12" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q12" s="2" t="s">
+      <c r="Q12" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="R12" s="2" t="s">
+      <c r="R12" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="S12" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T12" s="3">
+      <c r="S12" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T12" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="13" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="2" t="s">
+      <c r="A13" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="D13" s="2" t="s">
+      <c r="D13" s="1" t="s">
         <v>110</v>
       </c>
       <c r="E13" s="1">
@@ -1934,39 +1928,39 @@
       <c r="M13" s="1">
         <v>131072</v>
       </c>
-      <c r="N13" s="2" t="s">
+      <c r="N13" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="O13" s="2" t="s">
+      <c r="O13" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="P13" s="2" t="s">
+      <c r="P13" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q13" s="2" t="s">
+      <c r="Q13" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="R13" s="2" t="s">
+      <c r="R13" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="S13" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T13" s="3">
+      <c r="S13" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T13" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="14" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="D14" s="2" t="s">
+      <c r="D14" s="1" t="s">
         <v>111</v>
       </c>
       <c r="E14" s="1">
@@ -1996,39 +1990,39 @@
       <c r="M14" s="1">
         <v>131072</v>
       </c>
-      <c r="N14" s="2" t="s">
+      <c r="N14" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="O14" s="2" t="s">
+      <c r="O14" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="P14" s="2" t="s">
+      <c r="P14" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q14" s="2" t="s">
+      <c r="Q14" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="R14" s="2" t="s">
+      <c r="R14" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="S14" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T14" s="3">
+      <c r="S14" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T14" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="15" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D15" s="2" t="s">
+      <c r="D15" s="1" t="s">
         <v>114</v>
       </c>
       <c r="E15" s="1">
@@ -2058,39 +2052,39 @@
       <c r="M15" s="1">
         <v>128000</v>
       </c>
-      <c r="N15" s="2" t="s">
+      <c r="N15" s="1" t="s">
         <v>115</v>
       </c>
-      <c r="O15" s="2" t="s">
+      <c r="O15" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="P15" s="2" t="s">
+      <c r="P15" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q15" s="2" t="s">
+      <c r="Q15" s="1" t="s">
         <v>117</v>
       </c>
-      <c r="R15" s="2" t="s">
+      <c r="R15" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="S15" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T15" s="3">
+      <c r="S15" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T15" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
     <row r="16" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="2" t="s">
+      <c r="A16" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D16" s="2" t="s">
+      <c r="D16" s="1" t="s">
         <v>118</v>
       </c>
       <c r="E16" s="1">
@@ -2120,25 +2114,25 @@
       <c r="M16" s="1">
         <v>131072</v>
       </c>
-      <c r="N16" s="2" t="s">
+      <c r="N16" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="O16" s="2" t="s">
+      <c r="O16" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="P16" s="2" t="s">
+      <c r="P16" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="Q16" s="2" t="s">
+      <c r="Q16" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="R16" s="2" t="s">
+      <c r="R16" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="S16" s="3">
-        <v>46031.317484479165</v>
-      </c>
-      <c r="T16" s="3">
+      <c r="S16" s="2">
+        <v>46031.317484479165</v>
+      </c>
+      <c r="T16" s="2">
         <v>46031.317484479165</v>
       </c>
     </row>
@@ -2337,8 +2331,6 @@
       <c r="C4" s="1" t="s">
         <v>136</v>
       </c>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
       <c r="G4" s="1" t="s">
         <v>147</v>
       </c>

</xml_diff>

<commit_message>
update model analysis with feedback
</commit_message>
<xml_diff>
--- a/artifacts/analysis/model-analysis.xlsx
+++ b/artifacts/analysis/model-analysis.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jn\dev\llm-ensemble\artifacts\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{F9F8E4FD-DABA-4385-9460-4E76E1883B12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A1D622B-BE1C-47FE-9B6D-9D699A8D3D92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{D1A87F95-65CE-44FE-B65A-B20AE0988E6A}"/>
   </bookViews>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="184">
   <si>
     <t>model_id</t>
   </si>
@@ -604,6 +604,24 @@
   </si>
   <si>
     <t>Public and curated educational text and code; synthetic textbook-style learning data; human-labeled chat data; image–text interleaved data; public and synthetic image/video data; anonymized speech–text data; task-supervised speech data; synthetic speech data; synthetic vision–speech data</t>
+  </si>
+  <si>
+    <t>GUI Screenshots, Interaction Traces, Tutorials, Synthetic Data (iterative training with reflective online traces)</t>
+  </si>
+  <si>
+    <t>Web Documents, code, technical literature</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>slow</t>
+  </si>
+  <si>
+    <t>context too small</t>
+  </si>
+  <si>
+    <t>internal server error</t>
   </si>
 </sst>
 </file>
@@ -611,9 +629,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="[$-409]d\-mmm\-yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -634,8 +652,22 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C5700"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -645,6 +677,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -657,11 +699,13 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -672,50 +716,64 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="3" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="169" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="4">
+    <cellStyle name="Bad" xfId="2" builtinId="27"/>
     <cellStyle name="Good" xfId="1" builtinId="26"/>
+    <cellStyle name="Neutral" xfId="3" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="38">
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="169" formatCode="[$-409]d\-mmm\-yyyy;@"/>
+  <dxfs count="39">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy;@"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -765,6 +823,9 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -856,14 +917,14 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E74BC6F4-E459-4841-A57F-F7392AD4352B}" name="models_202601091237" displayName="models_202601091237" ref="A1:T16" tableType="queryTable" totalsRowShown="0" headerRowDxfId="37" dataDxfId="36">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E74BC6F4-E459-4841-A57F-F7392AD4352B}" name="models_202601091237" displayName="models_202601091237" ref="A1:T16" tableType="queryTable" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <autoFilter ref="A1:T16" xr:uid="{E74BC6F4-E459-4841-A57F-F7392AD4352B}"/>
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{78D3B969-8519-472B-B7DC-40B2AB389EDF}" uniqueName="1" name="model_id" queryTableFieldId="1" dataDxfId="35"/>
-    <tableColumn id="2" xr3:uid="{2775870E-97E4-4A13-8631-08858414ABE9}" uniqueName="2" name="canonical_slug" queryTableFieldId="2" dataDxfId="34"/>
-    <tableColumn id="3" xr3:uid="{9123C448-65CD-42A3-A8DF-FA33362CF2EB}" uniqueName="3" name="model_name" queryTableFieldId="3" dataDxfId="33"/>
-    <tableColumn id="4" xr3:uid="{23ACEE67-B62B-4941-8C62-48ACD4FFD384}" uniqueName="4" name="description" queryTableFieldId="4" dataDxfId="32"/>
-    <tableColumn id="5" xr3:uid="{EBBFCEC0-7D31-4CAD-A2DD-E444E8C840AD}" uniqueName="5" name="created" queryTableFieldId="5" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{78D3B969-8519-472B-B7DC-40B2AB389EDF}" uniqueName="1" name="model_id" queryTableFieldId="1" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{2775870E-97E4-4A13-8631-08858414ABE9}" uniqueName="2" name="canonical_slug" queryTableFieldId="2" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{9123C448-65CD-42A3-A8DF-FA33362CF2EB}" uniqueName="3" name="model_name" queryTableFieldId="3" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{23ACEE67-B62B-4941-8C62-48ACD4FFD384}" uniqueName="4" name="description" queryTableFieldId="4" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{EBBFCEC0-7D31-4CAD-A2DD-E444E8C840AD}" uniqueName="5" name="created" queryTableFieldId="5" dataDxfId="32"/>
     <tableColumn id="6" xr3:uid="{235BBD11-52A4-432B-B259-1FEF7849A476}" uniqueName="6" name="prompt_cost_per_1m" queryTableFieldId="6" dataDxfId="31"/>
     <tableColumn id="7" xr3:uid="{C125A326-71DC-498F-9CF6-9D4261986ABF}" uniqueName="7" name="completion_cost_per_1m" queryTableFieldId="7" dataDxfId="30"/>
     <tableColumn id="8" xr3:uid="{C48D515D-EA76-4B8D-9D9B-3F86005C986D}" uniqueName="8" name="avg_cost_per_1m" queryTableFieldId="8" dataDxfId="29"/>
@@ -885,23 +946,24 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2515506D-7B69-4B06-9BF5-773B122E6626}" name="Table6" displayName="Table6" ref="A1:N16" totalsRowShown="0" headerRowDxfId="1" dataDxfId="0" headerRowCellStyle="Normal" dataCellStyle="Normal">
-  <autoFilter ref="A1:N16" xr:uid="{2515506D-7B69-4B06-9BF5-773B122E6626}"/>
-  <tableColumns count="14">
-    <tableColumn id="1" xr3:uid="{D58B9424-3D3A-43E3-A095-F707C822ADC7}" name="model_id" dataDxfId="15" dataCellStyle="Normal"/>
-    <tableColumn id="2" xr3:uid="{00B31618-54C8-49F9-A9FF-AA301F6B83EE}" name="provider" dataDxfId="14" dataCellStyle="Normal"/>
-    <tableColumn id="15" xr3:uid="{B2A402DF-F928-46BF-A6E6-444AE9EAEC05}" name="Location" dataDxfId="13" dataCellStyle="Normal"/>
-    <tableColumn id="9" xr3:uid="{7B44B058-78D5-4162-B76D-3974F66C0617}" name="Parameter size" dataDxfId="12" dataCellStyle="Normal"/>
-    <tableColumn id="10" xr3:uid="{E2191CB7-B6FF-404B-9962-2076D050CEB7}" name="context_length" dataDxfId="11" dataCellStyle="Normal"/>
-    <tableColumn id="11" xr3:uid="{521CF197-E079-4F72-80B5-C09DE2953B51}" name="avg_cost_per_1m" dataDxfId="10" dataCellStyle="Normal"/>
-    <tableColumn id="16" xr3:uid="{68946881-DC74-4AD2-8B91-5A1883D0EBA1}" name="Release Date" dataDxfId="9" dataCellStyle="Good"/>
-    <tableColumn id="3" xr3:uid="{FB0B91F9-CC4A-4F2F-B7FA-8F4849679D55}" name="training data" dataDxfId="8" dataCellStyle="Normal"/>
-    <tableColumn id="4" xr3:uid="{710908A7-2136-47EA-9EA4-61FB50EB1236}" name="Input modalities" dataDxfId="7" dataCellStyle="Normal"/>
-    <tableColumn id="5" xr3:uid="{E231CFF8-225F-4DDB-B084-555A9DCA2D9B}" name="Output modalities" dataDxfId="6" dataCellStyle="Normal"/>
-    <tableColumn id="7" xr3:uid="{ACE0B5AB-F0DE-44AF-BDA1-3D7933AA8AF9}" name="Reasoning" dataDxfId="5" dataCellStyle="Normal"/>
-    <tableColumn id="8" xr3:uid="{81A13497-D9E5-4952-BA69-5ECB2716882B}" name="Use Case" dataDxfId="4" dataCellStyle="Normal"/>
-    <tableColumn id="12" xr3:uid="{2143AF97-E365-40D2-8B0E-2F9755C0F893}" name="openrouter link" dataDxfId="3" dataCellStyle="Normal"/>
-    <tableColumn id="13" xr3:uid="{0516A28C-43F7-4683-AB8C-D7BCE4C57A35}" name="other links" dataDxfId="2" dataCellStyle="Normal"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2515506D-7B69-4B06-9BF5-773B122E6626}" name="Table6" displayName="Table6" ref="A1:O16" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" headerRowCellStyle="Normal" dataCellStyle="Normal">
+  <autoFilter ref="A1:O16" xr:uid="{2515506D-7B69-4B06-9BF5-773B122E6626}"/>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{D58B9424-3D3A-43E3-A095-F707C822ADC7}" name="model_id" dataDxfId="14" dataCellStyle="Normal"/>
+    <tableColumn id="2" xr3:uid="{00B31618-54C8-49F9-A9FF-AA301F6B83EE}" name="provider" dataDxfId="13" dataCellStyle="Normal"/>
+    <tableColumn id="15" xr3:uid="{B2A402DF-F928-46BF-A6E6-444AE9EAEC05}" name="Location" dataDxfId="12" dataCellStyle="Normal"/>
+    <tableColumn id="9" xr3:uid="{7B44B058-78D5-4162-B76D-3974F66C0617}" name="Parameter size" dataDxfId="11" dataCellStyle="Normal"/>
+    <tableColumn id="10" xr3:uid="{E2191CB7-B6FF-404B-9962-2076D050CEB7}" name="context_length" dataDxfId="10" dataCellStyle="Normal"/>
+    <tableColumn id="11" xr3:uid="{521CF197-E079-4F72-80B5-C09DE2953B51}" name="avg_cost_per_1m" dataDxfId="9" dataCellStyle="Normal"/>
+    <tableColumn id="16" xr3:uid="{68946881-DC74-4AD2-8B91-5A1883D0EBA1}" name="Release Date" dataDxfId="8" dataCellStyle="Good"/>
+    <tableColumn id="3" xr3:uid="{FB0B91F9-CC4A-4F2F-B7FA-8F4849679D55}" name="training data" dataDxfId="7" dataCellStyle="Normal"/>
+    <tableColumn id="4" xr3:uid="{710908A7-2136-47EA-9EA4-61FB50EB1236}" name="Input modalities" dataDxfId="6" dataCellStyle="Normal"/>
+    <tableColumn id="5" xr3:uid="{E231CFF8-225F-4DDB-B084-555A9DCA2D9B}" name="Output modalities" dataDxfId="5" dataCellStyle="Normal"/>
+    <tableColumn id="7" xr3:uid="{ACE0B5AB-F0DE-44AF-BDA1-3D7933AA8AF9}" name="Reasoning" dataDxfId="4" dataCellStyle="Normal"/>
+    <tableColumn id="8" xr3:uid="{81A13497-D9E5-4952-BA69-5ECB2716882B}" name="Use Case" dataDxfId="3" dataCellStyle="Normal"/>
+    <tableColumn id="12" xr3:uid="{2143AF97-E365-40D2-8B0E-2F9755C0F893}" name="openrouter link" dataDxfId="2" dataCellStyle="Normal"/>
+    <tableColumn id="13" xr3:uid="{0516A28C-43F7-4683-AB8C-D7BCE4C57A35}" name="other links" dataDxfId="1" dataCellStyle="Normal"/>
+    <tableColumn id="6" xr3:uid="{A32E4A17-CBEB-4B4E-82ED-3C03A0E0104C}" name="note" dataDxfId="0" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2312,7 +2374,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ADB490E-EB07-4EE4-BECE-4EE10CDDA4E5}">
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr defaultRowHeight="40" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="33.90625" style="1" bestFit="1" customWidth="1"/>
@@ -2332,7 +2394,7 @@
     <col min="15" max="16384" width="8.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2351,7 +2413,7 @@
       <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="4" t="s">
         <v>166</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -2375,8 +2437,11 @@
       <c r="N1" s="1" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="2" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="O1" s="8" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>10</v>
       </c>
@@ -2395,8 +2460,11 @@
       <c r="F2" s="1">
         <v>0.15</v>
       </c>
-      <c r="G2" s="5">
+      <c r="G2" s="4">
         <v>45860.725185185191</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>178</v>
       </c>
       <c r="I2" s="1" t="s">
         <v>131</v>
@@ -2410,8 +2478,9 @@
       <c r="N2" s="1" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="3" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="O2" s="8"/>
+    </row>
+    <row r="3" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -2430,8 +2499,11 @@
       <c r="F3" s="1">
         <v>9.375E-2</v>
       </c>
-      <c r="G3" s="5">
+      <c r="G3" s="4">
         <v>45640.274907407409</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>179</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>49</v>
@@ -2445,8 +2517,9 @@
       <c r="M3" s="1" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="4" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="O3" s="8"/>
+    </row>
+    <row r="4" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -2465,7 +2538,7 @@
       <c r="F4" s="1">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="G4" s="5">
+      <c r="G4" s="4">
         <v>45806.714618055557</v>
       </c>
       <c r="K4" s="1" t="b">
@@ -2474,46 +2547,50 @@
       <c r="M4" s="1" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="5" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1" t="s">
+      <c r="O4" s="8"/>
+    </row>
+    <row r="5" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="D5" s="1">
+      <c r="D5" s="3">
         <v>4</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="3">
         <v>96000</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5" s="3">
         <v>4.2591860000000002E-2</v>
       </c>
       <c r="G5" s="5">
         <v>45729.943402777775</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="K5" s="3"/>
+      <c r="L5" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="M5" s="1" t="s">
+      <c r="M5" s="3" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="6" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="N5" s="3"/>
+      <c r="O5" s="3"/>
+    </row>
+    <row r="6" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>52</v>
       </c>
@@ -2532,7 +2609,7 @@
       <c r="F6" s="1">
         <v>6.3500000000000001E-2</v>
       </c>
-      <c r="G6" s="5">
+      <c r="G6" s="4">
         <v>45950.107581018514</v>
       </c>
       <c r="H6" s="1" t="s">
@@ -2547,8 +2624,9 @@
       <c r="M6" s="1" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="7" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="O6" s="8"/>
+    </row>
+    <row r="7" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>18</v>
       </c>
@@ -2567,7 +2645,7 @@
       <c r="F7" s="1">
         <v>0.04</v>
       </c>
-      <c r="G7" s="5">
+      <c r="G7" s="4">
         <v>45700.959699074076</v>
       </c>
       <c r="H7" s="1" t="s">
@@ -2585,49 +2663,54 @@
       <c r="M7" s="1" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="8" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="1" t="s">
+      <c r="O7" s="8"/>
+    </row>
+    <row r="8" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="D8" s="1">
+      <c r="D8" s="9">
         <v>3</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="9">
         <v>131072</v>
       </c>
-      <c r="F8" s="1">
+      <c r="F8" s="9">
         <v>0.02</v>
       </c>
-      <c r="G8" s="5">
+      <c r="G8" s="10">
         <v>45560</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="H8" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="I8" s="1" t="s">
+      <c r="I8" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="J8" s="1" t="s">
+      <c r="J8" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="L8" s="1" t="s">
+      <c r="K8" s="9"/>
+      <c r="L8" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="M8" s="1" t="s">
+      <c r="M8" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="N8" s="1" t="s">
+      <c r="N8" s="9" t="s">
         <v>121</v>
       </c>
-    </row>
-    <row r="9" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="O8" s="9" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>54</v>
       </c>
@@ -2646,7 +2729,7 @@
       <c r="F9" s="1">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="G9" s="5">
+      <c r="G9" s="4">
         <v>45724.049583333333</v>
       </c>
       <c r="H9" s="1" t="s">
@@ -2670,43 +2753,48 @@
       <c r="N9" s="1" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="10" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+      <c r="O9" s="8"/>
+    </row>
+    <row r="10" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="D10" s="1">
+      <c r="D10" s="3">
         <v>3</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="3">
         <v>131072</v>
       </c>
-      <c r="F10" s="1">
+      <c r="F10" s="3">
         <v>0.1</v>
       </c>
       <c r="G10" s="5">
         <v>45993.555092592593</v>
       </c>
-      <c r="I10" s="1" t="s">
+      <c r="H10" s="3"/>
+      <c r="I10" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="L10" s="1" t="s">
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+      <c r="L10" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="M10" s="1" t="s">
+      <c r="M10" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="N10" s="1" t="s">
+      <c r="N10" s="3" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="11" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="O10" s="3"/>
+    </row>
+    <row r="11" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
@@ -2725,7 +2813,7 @@
       <c r="F11" s="1">
         <v>0.15</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="4">
         <v>45993.556180555555</v>
       </c>
       <c r="I11" s="1" t="s">
@@ -2737,8 +2825,9 @@
       <c r="M11" s="1" t="s">
         <v>142</v>
       </c>
-    </row>
-    <row r="12" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="O11" s="8"/>
+    </row>
+    <row r="12" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
         <v>26</v>
       </c>
@@ -2757,18 +2846,18 @@
       <c r="F12" s="1">
         <v>0.04</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="4">
         <v>45582</v>
       </c>
-      <c r="H12" s="4"/>
       <c r="L12" s="1" t="s">
         <v>175</v>
       </c>
       <c r="M12" s="1" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="13" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="O12" s="8"/>
+    </row>
+    <row r="13" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>28</v>
       </c>
@@ -2787,7 +2876,7 @@
       <c r="F13" s="1">
         <v>0.1</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="4">
         <v>45582</v>
       </c>
       <c r="L13" s="1" t="s">
@@ -2796,132 +2885,143 @@
       <c r="M13" s="1" t="s">
         <v>144</v>
       </c>
-    </row>
-    <row r="14" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="1" t="s">
+      <c r="O13" s="8"/>
+    </row>
+    <row r="14" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="D14" s="1">
+      <c r="D14" s="9">
         <v>9</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="9">
         <v>131072</v>
       </c>
-      <c r="F14" s="1">
+      <c r="F14" s="9">
         <v>0.1</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G14" s="10">
         <v>45905.884340277778</v>
       </c>
-      <c r="I14" s="1" t="s">
+      <c r="H14" s="9"/>
+      <c r="I14" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="J14" s="1" t="s">
+      <c r="J14" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="K14" s="1" t="b">
+      <c r="K14" s="9" t="b">
         <v>1</v>
       </c>
-      <c r="L14" s="1" t="s">
+      <c r="L14" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="M14" s="1" t="s">
+      <c r="M14" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="N14" s="1" t="s">
+      <c r="N14" s="9" t="s">
         <v>151</v>
       </c>
-    </row>
-    <row r="15" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="3" t="s">
+      <c r="O14" s="9" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="6" t="s">
         <v>161</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="D15" s="3">
+      <c r="D15" s="6">
         <v>8</v>
       </c>
-      <c r="E15" s="3">
+      <c r="E15" s="6">
         <v>128000</v>
       </c>
-      <c r="F15" s="3">
+      <c r="F15" s="6">
         <v>8.6499999999999994E-2</v>
       </c>
-      <c r="G15" s="6">
+      <c r="G15" s="7">
         <v>45775.905462962968</v>
       </c>
-      <c r="H15" s="3" t="s">
+      <c r="H15" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="I15" s="3" t="s">
+      <c r="I15" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="J15" s="3" t="s">
+      <c r="J15" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="K15" s="3" t="b">
+      <c r="K15" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="L15" s="3" t="s">
+      <c r="L15" s="6" t="s">
         <v>158</v>
       </c>
-      <c r="M15" s="3" t="s">
+      <c r="M15" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="N15" s="3"/>
-    </row>
-    <row r="16" spans="1:14" s="1" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="1" t="s">
+      <c r="N15" s="6"/>
+      <c r="O15" s="8" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="6" t="s">
         <v>160</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="D16" s="1">
+      <c r="D16" s="6">
         <v>8</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="6">
         <v>131072</v>
       </c>
-      <c r="F16" s="1">
+      <c r="F16" s="6">
         <v>0.28999999999999998</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G16" s="7">
         <v>45944.732731481483</v>
       </c>
-      <c r="H16" s="1" t="s">
+      <c r="H16" s="6" t="s">
         <v>159</v>
       </c>
-      <c r="I16" s="1" t="s">
+      <c r="I16" s="6" t="s">
         <v>153</v>
       </c>
-      <c r="J16" s="1" t="s">
+      <c r="J16" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="K16" s="1" t="b">
+      <c r="K16" s="6" t="b">
         <v>1</v>
       </c>
-      <c r="L16" s="1" t="s">
+      <c r="L16" s="6" t="s">
         <v>154</v>
       </c>
-      <c r="M16" s="1" t="s">
+      <c r="M16" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="N16" s="1" t="s">
+      <c r="N16" s="6" t="s">
         <v>147</v>
+      </c>
+      <c r="O16" s="8" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
excel table to latex table script
</commit_message>
<xml_diff>
--- a/artifacts/analysis/model-analysis.xlsx
+++ b/artifacts/analysis/model-analysis.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\jn\dev\llm-ensemble\artifacts\analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AB76A9F-0EA9-4FEC-9684-168D98D3CC60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DAEB5CF-5599-4798-99D8-17AC953A6B13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{D1A87F95-65CE-44FE-B65A-B20AE0988E6A}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{D1A87F95-65CE-44FE-B65A-B20AE0988E6A}"/>
   </bookViews>
   <sheets>
-    <sheet name="openrouter-data" sheetId="4" r:id="rId1"/>
-    <sheet name="model-analysis" sheetId="6" r:id="rId2"/>
+    <sheet name="model-analysis" sheetId="6" r:id="rId1"/>
+    <sheet name="openrouter-data" sheetId="4" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="ExternalData_3" localSheetId="0" hidden="1">'openrouter-data'!$A$1:$T$16</definedName>
+    <definedName name="ExternalData_3" localSheetId="1" hidden="1">'openrouter-data'!$A$1:$T$16</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -57,7 +57,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="193">
   <si>
     <t>model_id</t>
   </si>
@@ -167,9 +167,6 @@
     <t>Qwen: Qwen3 VL 8B Instruct</t>
   </si>
   <si>
-    <t>provider</t>
-  </si>
-  <si>
     <t>Nvidia</t>
   </si>
   <si>
@@ -189,12 +186,6 @@
   </si>
   <si>
     <t>Cohere</t>
-  </si>
-  <si>
-    <t>training data</t>
-  </si>
-  <si>
-    <t>Input modalities</t>
   </si>
   <si>
     <t>Output modalities</t>
@@ -452,18 +443,9 @@
     <t>Location</t>
   </si>
   <si>
-    <t>China</t>
-  </si>
-  <si>
-    <t>Canada</t>
-  </si>
-  <si>
     <t>US</t>
   </si>
   <si>
-    <t>France</t>
-  </si>
-  <si>
     <t>multimodal vision-language</t>
   </si>
   <si>
@@ -567,12 +549,6 @@
   </si>
   <si>
     <t>faster, memory-efficient inference</t>
-  </si>
-  <si>
-    <t>Release Date</t>
-  </si>
-  <si>
-    <t>Parameter size</t>
   </si>
   <si>
     <t>https://openrouter.ai/cohere/command-r7b-12-2024</t>
@@ -622,6 +598,57 @@
   </si>
   <si>
     <t>internal server error</t>
+  </si>
+  <si>
+    <t>fast</t>
+  </si>
+  <si>
+    <t>lightning-fast, possibly lots of 0 scores thorugh</t>
+  </si>
+  <si>
+    <t>128k</t>
+  </si>
+  <si>
+    <t>131k</t>
+  </si>
+  <si>
+    <t>262k</t>
+  </si>
+  <si>
+    <t>release</t>
+  </si>
+  <si>
+    <t>CN</t>
+  </si>
+  <si>
+    <t>CA</t>
+  </si>
+  <si>
+    <t>FR</t>
+  </si>
+  <si>
+    <t>096k</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>Provider</t>
+  </si>
+  <si>
+    <t>ParamSize</t>
+  </si>
+  <si>
+    <t>CtxLength</t>
+  </si>
+  <si>
+    <t>Cost</t>
+  </si>
+  <si>
+    <t>Training Data</t>
+  </si>
+  <si>
+    <t>Input</t>
   </si>
 </sst>
 </file>
@@ -631,7 +658,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy;@"/>
   </numFmts>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -654,6 +681,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -667,7 +701,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -689,6 +723,12 @@
         <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -699,13 +739,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -722,23 +763,30 @@
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="3" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="3" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" xfId="3" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="2" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="2" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="0" xfId="2" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="4" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="0" xfId="4" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="4">
+  <cellStyles count="5">
+    <cellStyle name="60% - Accent5" xfId="4" builtinId="48"/>
     <cellStyle name="Bad" xfId="2" builtinId="27"/>
     <cellStyle name="Good" xfId="1" builtinId="26"/>
     <cellStyle name="Neutral" xfId="3" builtinId="28"/>
@@ -746,31 +794,31 @@
   </cellStyles>
   <dxfs count="39">
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="[$-409]d\-mmm\-yyyy;@"/>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -917,8 +965,38 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2515506D-7B69-4B06-9BF5-773B122E6626}" name="Table6" displayName="Table6" ref="A1:O16" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" headerRowCellStyle="Normal" dataCellStyle="Normal">
+  <autoFilter ref="A1:O16" xr:uid="{2515506D-7B69-4B06-9BF5-773B122E6626}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:O16">
+    <sortCondition ref="A1:A16"/>
+  </sortState>
+  <tableColumns count="15">
+    <tableColumn id="1" xr3:uid="{D58B9424-3D3A-43E3-A095-F707C822ADC7}" name="Model" dataDxfId="14" dataCellStyle="Normal"/>
+    <tableColumn id="2" xr3:uid="{00B31618-54C8-49F9-A9FF-AA301F6B83EE}" name="Provider" dataDxfId="13" dataCellStyle="Normal"/>
+    <tableColumn id="15" xr3:uid="{B2A402DF-F928-46BF-A6E6-444AE9EAEC05}" name="Location" dataDxfId="12" dataCellStyle="Normal"/>
+    <tableColumn id="9" xr3:uid="{7B44B058-78D5-4162-B76D-3974F66C0617}" name="ParamSize" dataDxfId="11" dataCellStyle="Normal"/>
+    <tableColumn id="10" xr3:uid="{E2191CB7-B6FF-404B-9962-2076D050CEB7}" name="CtxLength" dataDxfId="10" dataCellStyle="Normal"/>
+    <tableColumn id="11" xr3:uid="{521CF197-E079-4F72-80B5-C09DE2953B51}" name="Cost" dataDxfId="1" dataCellStyle="Normal"/>
+    <tableColumn id="14" xr3:uid="{A8A63267-BB5B-463C-8484-6D28406DE281}" name="release" dataDxfId="0" dataCellStyle="Neutral"/>
+    <tableColumn id="3" xr3:uid="{FB0B91F9-CC4A-4F2F-B7FA-8F4849679D55}" name="Training Data" dataDxfId="9" dataCellStyle="Normal"/>
+    <tableColumn id="4" xr3:uid="{710908A7-2136-47EA-9EA4-61FB50EB1236}" name="Input" dataDxfId="8" dataCellStyle="Normal"/>
+    <tableColumn id="5" xr3:uid="{E231CFF8-225F-4DDB-B084-555A9DCA2D9B}" name="Output modalities" dataDxfId="7" dataCellStyle="Normal"/>
+    <tableColumn id="7" xr3:uid="{ACE0B5AB-F0DE-44AF-BDA1-3D7933AA8AF9}" name="Reasoning" dataDxfId="6" dataCellStyle="Normal"/>
+    <tableColumn id="8" xr3:uid="{81A13497-D9E5-4952-BA69-5ECB2716882B}" name="Use Case" dataDxfId="5" dataCellStyle="Normal"/>
+    <tableColumn id="12" xr3:uid="{2143AF97-E365-40D2-8B0E-2F9755C0F893}" name="openrouter link" dataDxfId="4" dataCellStyle="Normal"/>
+    <tableColumn id="13" xr3:uid="{0516A28C-43F7-4683-AB8C-D7BCE4C57A35}" name="other links" dataDxfId="3" dataCellStyle="Normal"/>
+    <tableColumn id="6" xr3:uid="{A32E4A17-CBEB-4B4E-82ED-3C03A0E0104C}" name="note" dataDxfId="2" dataCellStyle="Normal"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E74BC6F4-E459-4841-A57F-F7392AD4352B}" name="models_202601091237" displayName="models_202601091237" ref="A1:T16" tableType="queryTable" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <autoFilter ref="A1:T16" xr:uid="{E74BC6F4-E459-4841-A57F-F7392AD4352B}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:T16">
+    <sortCondition ref="A1:A16"/>
+  </sortState>
   <tableColumns count="20">
     <tableColumn id="1" xr3:uid="{78D3B969-8519-472B-B7DC-40B2AB389EDF}" uniqueName="1" name="model_id" queryTableFieldId="1" dataDxfId="36"/>
     <tableColumn id="2" xr3:uid="{2775870E-97E4-4A13-8631-08858414ABE9}" uniqueName="2" name="canonical_slug" queryTableFieldId="2" dataDxfId="35"/>
@@ -942,30 +1020,6 @@
     <tableColumn id="20" xr3:uid="{A9E6322E-6414-4705-8C48-2E513F4761A1}" uniqueName="20" name="created_at" queryTableFieldId="20" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{2515506D-7B69-4B06-9BF5-773B122E6626}" name="Table6" displayName="Table6" ref="A1:O16" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15" headerRowCellStyle="Normal" dataCellStyle="Normal">
-  <autoFilter ref="A1:O16" xr:uid="{2515506D-7B69-4B06-9BF5-773B122E6626}"/>
-  <tableColumns count="15">
-    <tableColumn id="1" xr3:uid="{D58B9424-3D3A-43E3-A095-F707C822ADC7}" name="model_id" dataDxfId="14" dataCellStyle="Normal"/>
-    <tableColumn id="2" xr3:uid="{00B31618-54C8-49F9-A9FF-AA301F6B83EE}" name="provider" dataDxfId="13" dataCellStyle="Normal"/>
-    <tableColumn id="15" xr3:uid="{B2A402DF-F928-46BF-A6E6-444AE9EAEC05}" name="Location" dataDxfId="12" dataCellStyle="Normal"/>
-    <tableColumn id="9" xr3:uid="{7B44B058-78D5-4162-B76D-3974F66C0617}" name="Parameter size" dataDxfId="11" dataCellStyle="Normal"/>
-    <tableColumn id="10" xr3:uid="{E2191CB7-B6FF-404B-9962-2076D050CEB7}" name="context_length" dataDxfId="10" dataCellStyle="Normal"/>
-    <tableColumn id="11" xr3:uid="{521CF197-E079-4F72-80B5-C09DE2953B51}" name="avg_cost_per_1m" dataDxfId="9" dataCellStyle="Normal"/>
-    <tableColumn id="16" xr3:uid="{68946881-DC74-4AD2-8B91-5A1883D0EBA1}" name="Release Date" dataDxfId="8" dataCellStyle="Good"/>
-    <tableColumn id="3" xr3:uid="{FB0B91F9-CC4A-4F2F-B7FA-8F4849679D55}" name="training data" dataDxfId="7" dataCellStyle="Normal"/>
-    <tableColumn id="4" xr3:uid="{710908A7-2136-47EA-9EA4-61FB50EB1236}" name="Input modalities" dataDxfId="6" dataCellStyle="Normal"/>
-    <tableColumn id="5" xr3:uid="{E231CFF8-225F-4DDB-B084-555A9DCA2D9B}" name="Output modalities" dataDxfId="5" dataCellStyle="Normal"/>
-    <tableColumn id="7" xr3:uid="{ACE0B5AB-F0DE-44AF-BDA1-3D7933AA8AF9}" name="Reasoning" dataDxfId="4" dataCellStyle="Normal"/>
-    <tableColumn id="8" xr3:uid="{81A13497-D9E5-4952-BA69-5ECB2716882B}" name="Use Case" dataDxfId="3" dataCellStyle="Normal"/>
-    <tableColumn id="12" xr3:uid="{2143AF97-E365-40D2-8B0E-2F9755C0F893}" name="openrouter link" dataDxfId="2" dataCellStyle="Normal"/>
-    <tableColumn id="13" xr3:uid="{0516A28C-43F7-4683-AB8C-D7BCE4C57A35}" name="other links" dataDxfId="1" dataCellStyle="Normal"/>
-    <tableColumn id="6" xr3:uid="{A32E4A17-CBEB-4B4E-82ED-3C03A0E0104C}" name="note" dataDxfId="0" dataCellStyle="Normal"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1285,6 +1339,671 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ADB490E-EB07-4EE4-BECE-4EE10CDDA4E5}">
+  <dimension ref="A1:O16"/>
+  <sheetFormatPr defaultRowHeight="40" customHeight="1" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="33" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="9.90625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="7.1796875" style="1" customWidth="1"/>
+    <col min="7" max="7" width="19.1796875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="26.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.90625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.1796875" style="1" customWidth="1"/>
+    <col min="12" max="12" width="46.26953125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="77.36328125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="25.26953125" style="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.7265625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="O1" s="8" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="D2" s="1">
+        <v>7</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="F2" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="G2" s="4">
+        <v>45860.725185185191</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="O2" s="8"/>
+    </row>
+    <row r="3" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="D3" s="1">
+        <v>7</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="F3" s="1">
+        <v>9.375E-2</v>
+      </c>
+      <c r="G3" s="4">
+        <v>45640.274907407409</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="K3" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="M3" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="O3" s="8"/>
+    </row>
+    <row r="4" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="D4" s="1">
+        <v>8</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="F4" s="1">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G4" s="4">
+        <v>45806.714618055557</v>
+      </c>
+      <c r="K4" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="M4" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="O4" s="8"/>
+    </row>
+    <row r="5" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D5" s="3">
+        <v>4</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>185</v>
+      </c>
+      <c r="F5" s="3">
+        <v>4.2591860000000002E-2</v>
+      </c>
+      <c r="G5" s="5">
+        <v>45729.943402777775</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="K5" s="3"/>
+      <c r="L5" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="N5" s="3"/>
+      <c r="O5" s="3" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D6" s="1">
+        <v>3</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F6" s="1">
+        <v>6.3500000000000001E-2</v>
+      </c>
+      <c r="G6" s="4">
+        <v>45950.107581018514</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="O6" s="8"/>
+    </row>
+    <row r="7" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="D7" s="9">
+        <v>3</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="F7" s="9">
+        <v>0.02</v>
+      </c>
+      <c r="G7" s="10">
+        <v>45560</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="K7" s="9"/>
+      <c r="L7" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="M7" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="N7" s="9" t="s">
+        <v>118</v>
+      </c>
+      <c r="O7" s="9" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="D8" s="1">
+        <v>8</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F8" s="1">
+        <v>0.04</v>
+      </c>
+      <c r="G8" s="4">
+        <v>45700.959699074076</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="O8" s="8"/>
+    </row>
+    <row r="9" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>122</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="D9" s="11">
+        <v>6</v>
+      </c>
+      <c r="E9" s="11" t="s">
+        <v>179</v>
+      </c>
+      <c r="F9" s="11">
+        <v>7.4999999999999997E-2</v>
+      </c>
+      <c r="G9" s="12">
+        <v>45724.049583333333</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>169</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="J9" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="K9" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="L9" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="M9" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="N9" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="O9" s="11"/>
+    </row>
+    <row r="10" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D10" s="1">
+        <v>3</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0.04</v>
+      </c>
+      <c r="G10" s="4">
+        <v>45582</v>
+      </c>
+      <c r="H10" s="8"/>
+      <c r="L10" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="M10" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="O10" s="8"/>
+    </row>
+    <row r="11" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="D11" s="3">
+        <v>3</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="F11" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="G11" s="5">
+        <v>45993.555092592593</v>
+      </c>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+      <c r="L11" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="M11" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="N11" s="3" t="s">
+        <v>157</v>
+      </c>
+      <c r="O11" s="3" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D12" s="1">
+        <v>8</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F12" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="G12" s="4">
+        <v>45582</v>
+      </c>
+      <c r="L12" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="M12" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="O12" s="8"/>
+    </row>
+    <row r="13" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="D13" s="1">
+        <v>8</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="G13" s="4">
+        <v>45993.556180555555</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="L13" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="M13" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="O13" s="8"/>
+    </row>
+    <row r="14" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="D14" s="9">
+        <v>9</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>179</v>
+      </c>
+      <c r="F14" s="9">
+        <v>0.1</v>
+      </c>
+      <c r="G14" s="10">
+        <v>45905.884340277778</v>
+      </c>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="J14" s="9" t="s">
+        <v>129</v>
+      </c>
+      <c r="K14" s="9" t="b">
+        <v>1</v>
+      </c>
+      <c r="L14" s="9" t="s">
+        <v>143</v>
+      </c>
+      <c r="M14" s="9" t="s">
+        <v>146</v>
+      </c>
+      <c r="N14" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="O14" s="9" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="6" t="s">
+        <v>155</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="D15" s="6">
+        <v>8</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>178</v>
+      </c>
+      <c r="F15" s="6">
+        <v>8.6499999999999994E-2</v>
+      </c>
+      <c r="G15" s="7">
+        <v>45775.905462962968</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="K15" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="L15" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="M15" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="N15" s="6"/>
+      <c r="O15" s="6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>182</v>
+      </c>
+      <c r="D16" s="6">
+        <v>8</v>
+      </c>
+      <c r="E16" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="F16" s="6">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="G16" s="7">
+        <v>45944.732731481483</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>153</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>129</v>
+      </c>
+      <c r="K16" s="6" t="b">
+        <v>1</v>
+      </c>
+      <c r="L16" s="6" t="s">
+        <v>148</v>
+      </c>
+      <c r="M16" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="N16" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="O16" s="6" t="s">
+        <v>173</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{030068A6-33CF-4092-B5E5-65A22CC450D3}">
   <dimension ref="A1:T26"/>
   <sheetFormatPr defaultRowHeight="40" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -1316,16 +2035,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="F1" s="1" t="s">
         <v>2</v>
@@ -1337,10 +2056,10 @@
         <v>4</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="K1" s="1" t="s">
         <v>5</v>
@@ -1352,19 +2071,19 @@
         <v>7</v>
       </c>
       <c r="N1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="Q1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>65</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>8</v>
@@ -1384,7 +2103,7 @@
         <v>11</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E2" s="1">
         <v>1753205056</v>
@@ -1414,19 +2133,19 @@
         <v>128000</v>
       </c>
       <c r="N2" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="P2" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q2" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="O2" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="P2" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q2" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="R2" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="S2" s="2">
         <v>46031.317484479165</v>
@@ -1446,7 +2165,7 @@
         <v>13</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E3" s="1">
         <v>1734158152</v>
@@ -1476,19 +2195,19 @@
         <v>128000</v>
       </c>
       <c r="N3" s="1" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="O3" s="1" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="R3" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="S3" s="2">
         <v>46031.317484479165</v>
@@ -1508,7 +2227,7 @@
         <v>15</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E4" s="1">
         <v>1748538543</v>
@@ -1538,19 +2257,19 @@
         <v>128000</v>
       </c>
       <c r="N4" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="O4" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="R4" s="1" t="s">
         <v>76</v>
-      </c>
-      <c r="O4" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="P4" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q4" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="R4" s="1" t="s">
-        <v>79</v>
       </c>
       <c r="S4" s="2">
         <v>46031.317484479165</v>
@@ -1570,7 +2289,7 @@
         <v>17</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="E5" s="1">
         <v>1741905510</v>
@@ -1600,19 +2319,19 @@
         <v>96000</v>
       </c>
       <c r="N5" s="1" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="O5" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="R5" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="S5" s="2">
         <v>46031.317484479165</v>
@@ -1623,16 +2342,16 @@
     </row>
     <row r="6" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="E6" s="1">
         <v>1760927695</v>
@@ -1662,19 +2381,19 @@
         <v>131000</v>
       </c>
       <c r="N6" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="O6" s="1" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="R6" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="S6" s="2">
         <v>46031.317484479165</v>
@@ -1685,28 +2404,28 @@
     </row>
     <row r="7" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>88</v>
       </c>
       <c r="E7" s="1">
-        <v>1739401318</v>
+        <v>1727222400</v>
       </c>
       <c r="F7" s="1">
         <v>0.02</v>
       </c>
       <c r="G7" s="1">
-        <v>0.06</v>
+        <v>0.02</v>
       </c>
       <c r="H7" s="1">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="I7" s="1">
         <v>0</v>
@@ -1718,7 +2437,7 @@
         <v>0</v>
       </c>
       <c r="L7" s="1">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="M7" s="1">
         <v>131072</v>
@@ -1730,13 +2449,13 @@
         <v>90</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="R7" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="S7" s="2">
         <v>46031.317484479165</v>
@@ -1747,28 +2466,28 @@
     </row>
     <row r="8" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="E8" s="1">
-        <v>1727222400</v>
+        <v>1739401318</v>
       </c>
       <c r="F8" s="1">
         <v>0.02</v>
       </c>
       <c r="G8" s="1">
-        <v>0.02</v>
+        <v>0.06</v>
       </c>
       <c r="H8" s="1">
-        <v>0.02</v>
+        <v>0.04</v>
       </c>
       <c r="I8" s="1">
         <v>0</v>
@@ -1780,25 +2499,25 @@
         <v>0</v>
       </c>
       <c r="L8" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M8" s="1">
         <v>131072</v>
       </c>
       <c r="N8" s="1" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="O8" s="1" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="R8" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="S8" s="2">
         <v>46031.317484479165</v>
@@ -1809,16 +2528,16 @@
     </row>
     <row r="9" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E9" s="1">
         <v>1741396284</v>
@@ -1848,19 +2567,19 @@
         <v>131072</v>
       </c>
       <c r="N9" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="O9" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="R9" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="S9" s="2">
         <v>46031.317484479165</v>
@@ -1871,28 +2590,28 @@
     </row>
     <row r="10" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="E10" s="1">
-        <v>1764681560</v>
+        <v>1729123200</v>
       </c>
       <c r="F10" s="1">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="G10" s="1">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="H10" s="1">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="I10" s="1">
         <v>0</v>
@@ -1910,19 +2629,19 @@
         <v>131072</v>
       </c>
       <c r="N10" s="1" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="O10" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="R10" s="1" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="S10" s="2">
         <v>46031.317484479165</v>
@@ -1933,28 +2652,28 @@
     </row>
     <row r="11" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="E11" s="1">
-        <v>1764681654</v>
+        <v>1764681560</v>
       </c>
       <c r="F11" s="1">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="G11" s="1">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="H11" s="1">
-        <v>0.15</v>
+        <v>0.1</v>
       </c>
       <c r="I11" s="1">
         <v>0</v>
@@ -1966,25 +2685,25 @@
         <v>0</v>
       </c>
       <c r="L11" s="1">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="M11" s="1">
-        <v>262144</v>
+        <v>131072</v>
       </c>
       <c r="N11" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="O11" s="1" t="s">
-        <v>102</v>
+        <v>87</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="R11" s="1" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="S11" s="2">
         <v>46031.317484479165</v>
@@ -1995,13 +2714,13 @@
     </row>
     <row r="12" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>103</v>
@@ -2010,13 +2729,13 @@
         <v>1729123200</v>
       </c>
       <c r="F12" s="1">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="G12" s="1">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="H12" s="1">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="I12" s="1">
         <v>0</v>
@@ -2028,25 +2747,25 @@
         <v>0</v>
       </c>
       <c r="L12" s="1">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="M12" s="1">
         <v>131072</v>
       </c>
       <c r="N12" s="1" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="O12" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="R12" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="S12" s="2">
         <v>46031.317484479165</v>
@@ -2057,28 +2776,28 @@
     </row>
     <row r="13" spans="1:20" ht="40" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="E13" s="1">
-        <v>1729123200</v>
+        <v>1764681654</v>
       </c>
       <c r="F13" s="1">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="G13" s="1">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="H13" s="1">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="I13" s="1">
         <v>0</v>
@@ -2093,22 +2812,22 @@
         <v>8</v>
       </c>
       <c r="M13" s="1">
-        <v>131072</v>
+        <v>262144</v>
       </c>
       <c r="N13" s="1" t="s">
-        <v>104</v>
+        <v>95</v>
       </c>
       <c r="O13" s="1" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="S13" s="2">
         <v>46031.317484479165</v>
@@ -2128,7 +2847,7 @@
         <v>31</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="E14" s="1">
         <v>1757106807</v>
@@ -2158,19 +2877,19 @@
         <v>131072</v>
       </c>
       <c r="N14" s="1" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="O14" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Q14" s="1" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="R14" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="S14" s="2">
         <v>46031.317484479165</v>
@@ -2184,13 +2903,13 @@
         <v>32</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>33</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="E15" s="1">
         <v>1745876632</v>
@@ -2220,19 +2939,19 @@
         <v>128000</v>
       </c>
       <c r="N15" s="1" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="O15" s="1" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="Q15" s="1" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="S15" s="2">
         <v>46031.317484479165</v>
@@ -2252,7 +2971,7 @@
         <v>35</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="E16" s="1">
         <v>1760463308</v>
@@ -2282,19 +3001,19 @@
         <v>131072</v>
       </c>
       <c r="N16" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="O16" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="P16" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q16" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="R16" s="1" t="s">
         <v>115</v>
-      </c>
-      <c r="O16" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="P16" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="Q16" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="R16" s="1" t="s">
-        <v>118</v>
       </c>
       <c r="S16" s="2">
         <v>46031.317484479165</v>
@@ -2365,668 +3084,6 @@
       <c r="M26"/>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9ADB490E-EB07-4EE4-BECE-4EE10CDDA4E5}">
-  <dimension ref="A1:O16"/>
-  <sheetFormatPr defaultRowHeight="40" customHeight="1" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="33.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.90625" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.08984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.1796875" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="80" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="27.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22.7265625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.453125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="89.08984375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="47.36328125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="80" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.7265625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:15" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>167</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="O1" s="8" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D2" s="1">
-        <v>7</v>
-      </c>
-      <c r="E2" s="1">
-        <v>128000</v>
-      </c>
-      <c r="F2" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="G2" s="4">
-        <v>45860.725185185191</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>131</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>162</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>132</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>133</v>
-      </c>
-      <c r="O2" s="8"/>
-    </row>
-    <row r="3" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="D3" s="1">
-        <v>7</v>
-      </c>
-      <c r="E3" s="1">
-        <v>128000</v>
-      </c>
-      <c r="F3" s="1">
-        <v>9.375E-2</v>
-      </c>
-      <c r="G3" s="4">
-        <v>45640.274907407409</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>179</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="K3" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>157</v>
-      </c>
-      <c r="M3" s="1" t="s">
-        <v>168</v>
-      </c>
-      <c r="O3" s="8"/>
-    </row>
-    <row r="4" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="D4" s="1">
-        <v>8</v>
-      </c>
-      <c r="E4" s="1">
-        <v>128000</v>
-      </c>
-      <c r="F4" s="1">
-        <v>7.4999999999999997E-2</v>
-      </c>
-      <c r="G4" s="4">
-        <v>45806.714618055557</v>
-      </c>
-      <c r="K4" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="O4" s="8"/>
-    </row>
-    <row r="5" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D5" s="3">
-        <v>4</v>
-      </c>
-      <c r="E5" s="3">
-        <v>96000</v>
-      </c>
-      <c r="F5" s="3">
-        <v>4.2591860000000002E-2</v>
-      </c>
-      <c r="G5" s="5">
-        <v>45729.943402777775</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="K5" s="3"/>
-      <c r="L5" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="N5" s="3"/>
-      <c r="O5" s="3"/>
-    </row>
-    <row r="6" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="D6" s="1">
-        <v>3</v>
-      </c>
-      <c r="E6" s="1">
-        <v>131000</v>
-      </c>
-      <c r="F6" s="1">
-        <v>6.3500000000000001E-2</v>
-      </c>
-      <c r="G6" s="4">
-        <v>45950.107581018514</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="I6" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="M6" s="1" t="s">
-        <v>171</v>
-      </c>
-      <c r="O6" s="8"/>
-    </row>
-    <row r="7" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="D7" s="1">
-        <v>8</v>
-      </c>
-      <c r="E7" s="1">
-        <v>131072</v>
-      </c>
-      <c r="F7" s="1">
-        <v>0.04</v>
-      </c>
-      <c r="G7" s="4">
-        <v>45700.959699074076</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>156</v>
-      </c>
-      <c r="I7" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="O7" s="8"/>
-    </row>
-    <row r="8" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="D8" s="9">
-        <v>3</v>
-      </c>
-      <c r="E8" s="9">
-        <v>131072</v>
-      </c>
-      <c r="F8" s="9">
-        <v>0.02</v>
-      </c>
-      <c r="G8" s="10">
-        <v>45560</v>
-      </c>
-      <c r="H8" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="I8" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="J8" s="9" t="s">
-        <v>50</v>
-      </c>
-      <c r="K8" s="9"/>
-      <c r="L8" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="M8" s="9" t="s">
-        <v>120</v>
-      </c>
-      <c r="N8" s="9" t="s">
-        <v>121</v>
-      </c>
-      <c r="O8" s="9" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="9" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>129</v>
-      </c>
-      <c r="D9" s="1">
-        <v>5.6</v>
-      </c>
-      <c r="E9" s="1">
-        <v>131072</v>
-      </c>
-      <c r="F9" s="1">
-        <v>7.4999999999999997E-2</v>
-      </c>
-      <c r="G9" s="4">
-        <v>45724.049583333333</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>177</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>140</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>135</v>
-      </c>
-      <c r="K9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>139</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>173</v>
-      </c>
-      <c r="N9" s="1" t="s">
-        <v>176</v>
-      </c>
-      <c r="O9" s="8"/>
-    </row>
-    <row r="10" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D10" s="3">
-        <v>3</v>
-      </c>
-      <c r="E10" s="3">
-        <v>131072</v>
-      </c>
-      <c r="F10" s="3">
-        <v>0.1</v>
-      </c>
-      <c r="G10" s="5">
-        <v>45993.555092592593</v>
-      </c>
-      <c r="H10" s="3"/>
-      <c r="I10" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="J10" s="3"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="M10" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="N10" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="O10" s="3"/>
-    </row>
-    <row r="11" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D11" s="1">
-        <v>8</v>
-      </c>
-      <c r="E11" s="1">
-        <v>262144</v>
-      </c>
-      <c r="F11" s="1">
-        <v>0.15</v>
-      </c>
-      <c r="G11" s="4">
-        <v>45993.556180555555</v>
-      </c>
-      <c r="I11" s="1" t="s">
-        <v>148</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>164</v>
-      </c>
-      <c r="M11" s="1" t="s">
-        <v>142</v>
-      </c>
-      <c r="O11" s="8"/>
-    </row>
-    <row r="12" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D12" s="1">
-        <v>3</v>
-      </c>
-      <c r="E12" s="1">
-        <v>131072</v>
-      </c>
-      <c r="F12" s="1">
-        <v>0.04</v>
-      </c>
-      <c r="G12" s="4">
-        <v>45582</v>
-      </c>
-      <c r="H12" s="8"/>
-      <c r="L12" s="1" t="s">
-        <v>175</v>
-      </c>
-      <c r="M12" s="1" t="s">
-        <v>143</v>
-      </c>
-      <c r="O12" s="8"/>
-    </row>
-    <row r="13" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>130</v>
-      </c>
-      <c r="D13" s="1">
-        <v>8</v>
-      </c>
-      <c r="E13" s="1">
-        <v>131072</v>
-      </c>
-      <c r="F13" s="1">
-        <v>0.1</v>
-      </c>
-      <c r="G13" s="4">
-        <v>45582</v>
-      </c>
-      <c r="L13" s="1" t="s">
-        <v>165</v>
-      </c>
-      <c r="M13" s="1" t="s">
-        <v>144</v>
-      </c>
-      <c r="O13" s="8"/>
-    </row>
-    <row r="14" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A14" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>129</v>
-      </c>
-      <c r="D14" s="9">
-        <v>9</v>
-      </c>
-      <c r="E14" s="9">
-        <v>131072</v>
-      </c>
-      <c r="F14" s="9">
-        <v>0.1</v>
-      </c>
-      <c r="G14" s="10">
-        <v>45905.884340277778</v>
-      </c>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="J14" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="K14" s="9" t="b">
-        <v>1</v>
-      </c>
-      <c r="L14" s="9" t="s">
-        <v>149</v>
-      </c>
-      <c r="M14" s="9" t="s">
-        <v>152</v>
-      </c>
-      <c r="N14" s="9" t="s">
-        <v>151</v>
-      </c>
-      <c r="O14" s="9" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="15" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="6" t="s">
-        <v>161</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="D15" s="6">
-        <v>8</v>
-      </c>
-      <c r="E15" s="6">
-        <v>128000</v>
-      </c>
-      <c r="F15" s="6">
-        <v>8.6499999999999994E-2</v>
-      </c>
-      <c r="G15" s="7">
-        <v>45775.905462962968</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="I15" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="J15" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="K15" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="L15" s="6" t="s">
-        <v>158</v>
-      </c>
-      <c r="M15" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="N15" s="6"/>
-      <c r="O15" s="8" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="16" spans="1:15" ht="40" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>160</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="D16" s="6">
-        <v>8</v>
-      </c>
-      <c r="E16" s="6">
-        <v>131072</v>
-      </c>
-      <c r="F16" s="6">
-        <v>0.28999999999999998</v>
-      </c>
-      <c r="G16" s="7">
-        <v>45944.732731481483</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>159</v>
-      </c>
-      <c r="I16" s="6" t="s">
-        <v>153</v>
-      </c>
-      <c r="J16" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="K16" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="L16" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="M16" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="N16" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="O16" s="8" t="s">
-        <v>181</v>
-      </c>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>